<commit_message>
docs: actualiza documentación de la fase 3
</commit_message>
<xml_diff>
--- a/FASE 3/Documentacion del proyecto/MATRIZ CONTROL DE CAMBIO.xlsx
+++ b/FASE 3/Documentacion del proyecto/MATRIZ CONTROL DE CAMBIO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\clases 2022\Clases 2022-1\PTY4478\APT\Fase2_\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GAMER\CAPSTONE-PPY4614-007D\FASE 3\Documentacion del proyecto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92330C19-3FFC-4EB0-9ABA-74C33823D502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C709FF35-E060-45A9-86BF-629393DDE1A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14400" yWindow="0" windowWidth="14400" windowHeight="15600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="70">
   <si>
     <t>ID</t>
   </si>
@@ -90,13 +90,166 @@
   <si>
     <t>Aprobación:
 Aceptado-Rechazado</t>
+  </si>
+  <si>
+    <t>Equipo de desarrollo</t>
+  </si>
+  <si>
+    <t>Product Owner</t>
+  </si>
+  <si>
+    <t>Equipo UX</t>
+  </si>
+  <si>
+    <t>Equipo Machine Learning</t>
+  </si>
+  <si>
+    <t>Equipo QA</t>
+  </si>
+  <si>
+    <t>SC-07</t>
+  </si>
+  <si>
+    <t>SC-08</t>
+  </si>
+  <si>
+    <t>SC</t>
+  </si>
+  <si>
+    <t>Alta</t>
+  </si>
+  <si>
+    <t>Urgente</t>
+  </si>
+  <si>
+    <t>Migración de la base de datos</t>
+  </si>
+  <si>
+    <t>RF01: Gestión de datos del usuario</t>
+  </si>
+  <si>
+    <t>CU-03: Registrar emoción / CU-05: Consultar historial emocional</t>
+  </si>
+  <si>
+    <t>Desarrollo / Integración</t>
+  </si>
+  <si>
+    <t>Alto</t>
+  </si>
+  <si>
+    <t>Aceptado</t>
+  </si>
+  <si>
+    <t>Necesario</t>
+  </si>
+  <si>
+    <t>Solicitud de despliegue de la plataforma web en Render para disponibilidad pública y dominio accesible</t>
+  </si>
+  <si>
+    <t>RF-10: Acceso Web</t>
+  </si>
+  <si>
+    <t>CU-01: Iniciar Sesión / CU-02: Acceder al sistema</t>
+  </si>
+  <si>
+    <t>Despliegue</t>
+  </si>
+  <si>
+    <t>Medio</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>Media</t>
+  </si>
+  <si>
+    <t>Ajustes visuales en la App (paleta de colores, iconografía, mejoras de navegación)</t>
+  </si>
+  <si>
+    <t>RF-04: Interfaz de usuario amigable</t>
+  </si>
+  <si>
+    <t>CU-01: Iniciar sesión / CU-03: Registrar emoción</t>
+  </si>
+  <si>
+    <t>Construcción</t>
+  </si>
+  <si>
+    <t>Bajo</t>
+  </si>
+  <si>
+    <t>Crítico</t>
+  </si>
+  <si>
+    <t>Creación de un microservicio independiente para el modelo de recomendaciones con python</t>
+  </si>
+  <si>
+    <t>RF-07: Generación de recomendaciones personalizadas</t>
+  </si>
+  <si>
+    <t>CU-06: Obtener recomendaciones</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integración / Desarrollo </t>
+  </si>
+  <si>
+    <t>Solicitud de incorporar un chatbot funcional en la plataforma Desktop para acompañamiento básico</t>
+  </si>
+  <si>
+    <t>RF-08: Interacción conversacional</t>
+  </si>
+  <si>
+    <t>CU-07: Consultar chatbot</t>
+  </si>
+  <si>
+    <t>Desarrollo Desktop</t>
+  </si>
+  <si>
+    <t>Baja</t>
+  </si>
+  <si>
+    <t>Reprogramación del módulo administrativo web debido a limitaciones de tiempo del sprint</t>
+  </si>
+  <si>
+    <t>RF-11: Administración del sistema</t>
+  </si>
+  <si>
+    <t>CU-10: Gestionar usuarios</t>
+  </si>
+  <si>
+    <t>Validación</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Medio</t>
+  </si>
+  <si>
+    <t>Solicitud de incluir monitoreo del rendimiento de la API para estabilidad del sistema</t>
+  </si>
+  <si>
+    <t>RF-12: Monitoreo del sistema</t>
+  </si>
+  <si>
+    <t>CU-11: Verificar estado del backend</t>
+  </si>
+  <si>
+    <t>Implementación</t>
+  </si>
+  <si>
+    <t>Ajuste al modelo de datos para corregir inconsistencias en el historial emocional detectadas durante pruebas de integración</t>
+  </si>
+  <si>
+    <t>RF-01: Gestión de datos del usuario</t>
+  </si>
+  <si>
+    <t>CU-05: Consultar historial emocional</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -115,6 +268,12 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -187,30 +346,25 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -526,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.5703125" customWidth="1"/>
@@ -543,23 +697,23 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="9"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="9"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
     </row>
-    <row r="2" spans="1:12" s="6" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:12" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -568,148 +722,343 @@
       <c r="C2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="J2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="7" t="s">
+      <c r="K2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
+      <c r="B3" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="6">
+        <v>45935</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
+      <c r="B4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="6">
+        <v>45938</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
+      <c r="B5" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="6">
+        <v>45942</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
+      <c r="B6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="6">
+        <v>45948</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
+      <c r="B7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="6">
+        <v>45952</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
+      <c r="B8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="6">
+        <v>45955</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
+    <row r="9" spans="1:12" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="6">
+        <v>45958</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="90" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="6">
+        <v>45960</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:L1"/>
   </mergeCells>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967294" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>